<commit_message>
Update extensions, classes, table 28
minor edits based on file layout changes
</commit_message>
<xml_diff>
--- a/resources/property classes.xlsx
+++ b/resources/property classes.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28129"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cmapil-my.sharepoint.com/personal/abahls_cmap_illinois_gov/Documents/Documents/github_repos/effective_property_tax/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="13_ncr:1_{2A60A013-1040-4DEC-B76C-0C647DD12EE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BF013571-E9D9-4AA3-8254-A6847BA48987}"/>
+  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{2A60A013-1040-4DEC-B76C-0C647DD12EE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CB25FC7B-8658-46C7-B506-0720494CE9E0}"/>
   <bookViews>
-    <workbookView xWindow="17445" yWindow="-16320" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-11355" yWindow="-16365" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cook" sheetId="1" r:id="rId1"/>
@@ -23,8 +23,8 @@
     <sheet name="will" sheetId="7" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Cook!$A$1:$G$150</definedName>
-    <definedName name="Export_Output_2" localSheetId="0">Cook!$A$1:$E$134</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Cook!$A$1:$G$152</definedName>
+    <definedName name="Export_Output_2" localSheetId="0">Cook!$A$1:$E$136</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="932" uniqueCount="342">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="940" uniqueCount="343">
   <si>
     <t>overall_class</t>
   </si>
@@ -1071,6 +1071,9 @@
   </si>
   <si>
     <t>land_use_code</t>
+  </si>
+  <si>
+    <t>Commercial incentive land</t>
   </si>
 </sst>
 </file>
@@ -1440,7 +1443,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G150"/>
+  <dimension ref="A1:G152"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.44140625" bestFit="1" customWidth="1"/>
@@ -3038,7 +3041,7 @@
         <v>527</v>
       </c>
       <c r="B67" t="str">
-        <f t="shared" ref="B67:B130" si="1">TEXT(A67,"000")</f>
+        <f t="shared" ref="B67:B132" si="1">TEXT(A67,"000")</f>
         <v>527</v>
       </c>
       <c r="C67" t="s">
@@ -4331,14 +4334,14 @@
     </row>
     <row r="121" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A121">
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="B121" t="str">
         <f t="shared" si="1"/>
-        <v>801</v>
+        <v>800</v>
       </c>
       <c r="C121" t="s">
-        <v>121</v>
+        <v>342</v>
       </c>
       <c r="D121" t="s">
         <v>122</v>
@@ -4355,14 +4358,14 @@
     </row>
     <row r="122" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A122">
-        <v>817</v>
+        <v>801</v>
       </c>
       <c r="B122" t="str">
         <f t="shared" si="1"/>
-        <v>817</v>
+        <v>801</v>
       </c>
       <c r="C122" t="s">
-        <v>70</v>
+        <v>121</v>
       </c>
       <c r="D122" t="s">
         <v>122</v>
@@ -4379,14 +4382,14 @@
     </row>
     <row r="123" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A123">
-        <v>823</v>
+        <v>817</v>
       </c>
       <c r="B123" t="str">
         <f t="shared" si="1"/>
-        <v>823</v>
+        <v>817</v>
       </c>
       <c r="C123" t="s">
-        <v>124</v>
+        <v>70</v>
       </c>
       <c r="D123" t="s">
         <v>122</v>
@@ -4403,14 +4406,14 @@
     </row>
     <row r="124" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A124">
-        <v>827</v>
+        <v>823</v>
       </c>
       <c r="B124" t="str">
         <f t="shared" si="1"/>
-        <v>827</v>
+        <v>823</v>
       </c>
       <c r="C124" t="s">
-        <v>74</v>
+        <v>124</v>
       </c>
       <c r="D124" t="s">
         <v>122</v>
@@ -4427,14 +4430,14 @@
     </row>
     <row r="125" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A125">
-        <v>828</v>
+        <v>826</v>
       </c>
       <c r="B125" t="str">
         <f t="shared" si="1"/>
-        <v>828</v>
+        <v>826</v>
       </c>
       <c r="C125" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="D125" t="s">
         <v>122</v>
@@ -4451,14 +4454,14 @@
     </row>
     <row r="126" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A126">
-        <v>829</v>
+        <v>827</v>
       </c>
       <c r="B126" t="str">
         <f t="shared" si="1"/>
-        <v>829</v>
+        <v>827</v>
       </c>
       <c r="C126" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="D126" t="s">
         <v>122</v>
@@ -4475,14 +4478,14 @@
     </row>
     <row r="127" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A127">
-        <v>830</v>
+        <v>828</v>
       </c>
       <c r="B127" t="str">
         <f t="shared" si="1"/>
-        <v>830</v>
+        <v>828</v>
       </c>
       <c r="C127" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="D127" t="s">
         <v>122</v>
@@ -4499,14 +4502,14 @@
     </row>
     <row r="128" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A128">
-        <v>831</v>
+        <v>829</v>
       </c>
       <c r="B128" t="str">
         <f t="shared" si="1"/>
-        <v>831</v>
+        <v>829</v>
       </c>
       <c r="C128" t="s">
-        <v>125</v>
+        <v>76</v>
       </c>
       <c r="D128" t="s">
         <v>122</v>
@@ -4523,14 +4526,14 @@
     </row>
     <row r="129" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A129">
-        <v>833</v>
+        <v>830</v>
       </c>
       <c r="B129" t="str">
         <f t="shared" si="1"/>
-        <v>833</v>
+        <v>830</v>
       </c>
       <c r="C129" t="s">
-        <v>80</v>
+        <v>77</v>
       </c>
       <c r="D129" t="s">
         <v>122</v>
@@ -4547,17 +4550,17 @@
     </row>
     <row r="130" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A130">
-        <v>880</v>
+        <v>831</v>
       </c>
       <c r="B130" t="str">
         <f t="shared" si="1"/>
-        <v>880</v>
+        <v>831</v>
       </c>
       <c r="C130" t="s">
-        <v>85</v>
+        <v>125</v>
       </c>
       <c r="D130" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E130" t="s">
         <v>123</v>
@@ -4566,22 +4569,22 @@
         <v>0.101743</v>
       </c>
       <c r="G130" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
     </row>
     <row r="131" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A131">
-        <v>881</v>
+        <v>833</v>
       </c>
       <c r="B131" t="str">
-        <f t="shared" ref="B131:B150" si="2">TEXT(A131,"000")</f>
-        <v>881</v>
+        <f t="shared" si="1"/>
+        <v>833</v>
       </c>
       <c r="C131" t="s">
-        <v>105</v>
+        <v>80</v>
       </c>
       <c r="D131" t="s">
-        <v>126</v>
+        <v>122</v>
       </c>
       <c r="E131" t="s">
         <v>123</v>
@@ -4590,467 +4593,515 @@
         <v>0.101743</v>
       </c>
       <c r="G131" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
     </row>
     <row r="132" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A132">
+        <v>880</v>
+      </c>
+      <c r="B132" t="str">
+        <f t="shared" si="1"/>
+        <v>880</v>
+      </c>
+      <c r="C132" t="s">
+        <v>85</v>
+      </c>
+      <c r="D132" t="s">
+        <v>126</v>
+      </c>
+      <c r="E132" t="s">
+        <v>123</v>
+      </c>
+      <c r="F132">
+        <v>0.101743</v>
+      </c>
+      <c r="G132" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="133" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A133">
+        <v>881</v>
+      </c>
+      <c r="B133" t="str">
+        <f t="shared" ref="B133:B152" si="2">TEXT(A133,"000")</f>
+        <v>881</v>
+      </c>
+      <c r="C133" t="s">
+        <v>105</v>
+      </c>
+      <c r="D133" t="s">
+        <v>126</v>
+      </c>
+      <c r="E133" t="s">
+        <v>123</v>
+      </c>
+      <c r="F133">
+        <v>0.101743</v>
+      </c>
+      <c r="G133" t="s">
+        <v>157</v>
+      </c>
+    </row>
+    <row r="134" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A134">
         <v>883</v>
       </c>
-      <c r="B132" t="str">
+      <c r="B134" t="str">
         <f t="shared" si="2"/>
         <v>883</v>
       </c>
-      <c r="C132" t="s">
+      <c r="C134" t="s">
         <v>80</v>
       </c>
-      <c r="D132" t="s">
+      <c r="D134" t="s">
         <v>126</v>
       </c>
-      <c r="E132" t="s">
+      <c r="E134" t="s">
         <v>123</v>
       </c>
-      <c r="F132">
+      <c r="F134">
         <v>0.101743</v>
       </c>
-      <c r="G132" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="133" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A133">
+      <c r="G134" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="135" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A135">
         <v>887</v>
       </c>
-      <c r="B133" t="str">
+      <c r="B135" t="str">
         <f t="shared" si="2"/>
         <v>887</v>
       </c>
-      <c r="C133" t="s">
+      <c r="C135" t="s">
         <v>88</v>
       </c>
-      <c r="D133" t="s">
+      <c r="D135" t="s">
         <v>126</v>
       </c>
-      <c r="E133" t="s">
+      <c r="E135" t="s">
         <v>123</v>
       </c>
-      <c r="F133">
+      <c r="F135">
         <v>0.101743</v>
       </c>
-      <c r="G133" t="s">
+      <c r="G135" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="134" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A134">
+    <row r="136" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A136">
         <v>889</v>
       </c>
-      <c r="B134" t="str">
+      <c r="B136" t="str">
         <f t="shared" si="2"/>
         <v>889</v>
       </c>
-      <c r="C134" t="s">
+      <c r="C136" t="s">
         <v>89</v>
       </c>
-      <c r="D134" t="s">
+      <c r="D136" t="s">
         <v>126</v>
       </c>
-      <c r="E134" t="s">
+      <c r="E136" t="s">
         <v>123</v>
       </c>
-      <c r="F134">
+      <c r="F136">
         <v>0.101743</v>
       </c>
-      <c r="G134" t="s">
+      <c r="G136" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="135" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A135">
+    <row r="137" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A137">
         <v>890</v>
       </c>
-      <c r="B135" t="str">
+      <c r="B137" t="str">
         <f t="shared" si="2"/>
         <v>890</v>
       </c>
-      <c r="C135" t="s">
+      <c r="C137" t="s">
         <v>127</v>
       </c>
-      <c r="D135" t="s">
+      <c r="D137" t="s">
         <v>126</v>
       </c>
-      <c r="E135" t="s">
+      <c r="E137" t="s">
         <v>123</v>
       </c>
-      <c r="F135">
+      <c r="F137">
         <v>0.101743</v>
       </c>
-      <c r="G135" t="s">
+      <c r="G137" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="136" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A136">
+    <row r="138" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A138">
         <v>891</v>
       </c>
-      <c r="B136" t="str">
+      <c r="B138" t="str">
         <f t="shared" si="2"/>
         <v>891</v>
       </c>
-      <c r="C136" t="s">
+      <c r="C138" t="s">
         <v>117</v>
       </c>
-      <c r="D136" t="s">
+      <c r="D138" t="s">
         <v>122</v>
       </c>
-      <c r="E136" t="s">
+      <c r="E138" t="s">
         <v>123</v>
       </c>
-      <c r="F136">
+      <c r="F138">
         <v>0.101743</v>
       </c>
-      <c r="G136" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="137" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A137">
+      <c r="G138" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="139" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A139">
         <v>892</v>
       </c>
-      <c r="B137" t="str">
+      <c r="B139" t="str">
         <f t="shared" si="2"/>
         <v>892</v>
       </c>
-      <c r="C137" t="s">
+      <c r="C139" t="s">
         <v>92</v>
       </c>
-      <c r="D137" t="s">
+      <c r="D139" t="s">
         <v>122</v>
       </c>
-      <c r="E137" t="s">
+      <c r="E139" t="s">
         <v>123</v>
       </c>
-      <c r="F137">
+      <c r="F139">
         <v>0.101743</v>
       </c>
-      <c r="G137" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="138" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A138">
+      <c r="G139" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="140" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A140">
         <v>893</v>
       </c>
-      <c r="B138" t="str">
+      <c r="B140" t="str">
         <f t="shared" si="2"/>
         <v>893</v>
       </c>
-      <c r="C138" t="s">
+      <c r="C140" t="s">
         <v>93</v>
       </c>
-      <c r="D138" t="s">
+      <c r="D140" t="s">
         <v>126</v>
       </c>
-      <c r="E138" t="s">
+      <c r="E140" t="s">
         <v>123</v>
       </c>
-      <c r="F138">
+      <c r="F140">
         <v>0.101743</v>
       </c>
-      <c r="G138" t="s">
+      <c r="G140" t="s">
         <v>157</v>
       </c>
     </row>
-    <row r="139" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A139">
+    <row r="141" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A141">
         <v>897</v>
       </c>
-      <c r="B139" t="str">
+      <c r="B141" t="str">
         <f t="shared" si="2"/>
         <v>897</v>
       </c>
-      <c r="C139" t="s">
+      <c r="C141" t="s">
         <v>94</v>
       </c>
-      <c r="D139" t="s">
+      <c r="D141" t="s">
         <v>122</v>
       </c>
-      <c r="E139" t="s">
+      <c r="E141" t="s">
         <v>123</v>
       </c>
-      <c r="F139">
+      <c r="F141">
         <v>0.101743</v>
       </c>
-      <c r="G139" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="140" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A140">
+      <c r="G141" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="142" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A142">
         <v>899</v>
       </c>
-      <c r="B140" t="str">
+      <c r="B142" t="str">
         <f t="shared" si="2"/>
         <v>899</v>
       </c>
-      <c r="C140" t="s">
+      <c r="C142" t="s">
         <v>128</v>
       </c>
-      <c r="D140" t="s">
+      <c r="D142" t="s">
         <v>126</v>
       </c>
-      <c r="E140" t="s">
+      <c r="E142" t="s">
         <v>123</v>
       </c>
-      <c r="F140">
+      <c r="F142">
         <v>0.101743</v>
       </c>
-      <c r="G140" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="141" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A141">
+      <c r="G142" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="143" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A143">
         <v>900</v>
       </c>
-      <c r="B141" t="str">
+      <c r="B143" t="str">
         <f t="shared" si="2"/>
         <v>900</v>
       </c>
-      <c r="C141" t="s">
+      <c r="C143" t="s">
         <v>129</v>
       </c>
-      <c r="D141">
+      <c r="D143">
         <v>9</v>
       </c>
-      <c r="E141" t="s">
+      <c r="E143" t="s">
         <v>130</v>
       </c>
-      <c r="F141">
+      <c r="F143">
         <v>0.1</v>
       </c>
-      <c r="G141" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="142" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A142">
+      <c r="G143" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="144" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A144">
         <v>913</v>
       </c>
-      <c r="B142" t="str">
+      <c r="B144" t="str">
         <f t="shared" si="2"/>
         <v>913</v>
       </c>
-      <c r="C142" t="s">
+      <c r="C144" t="s">
         <v>131</v>
       </c>
-      <c r="D142">
+      <c r="D144">
         <v>9</v>
       </c>
-      <c r="E142" t="s">
+      <c r="E144" t="s">
         <v>130</v>
       </c>
-      <c r="F142">
+      <c r="F144">
         <v>0.1</v>
       </c>
-      <c r="G142" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="143" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A143">
+      <c r="G144" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="145" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A145">
         <v>914</v>
       </c>
-      <c r="B143" t="str">
+      <c r="B145" t="str">
         <f t="shared" si="2"/>
         <v>914</v>
       </c>
-      <c r="C143" t="s">
+      <c r="C145" t="s">
         <v>132</v>
       </c>
-      <c r="D143">
+      <c r="D145">
         <v>9</v>
       </c>
-      <c r="E143" t="s">
+      <c r="E145" t="s">
         <v>130</v>
       </c>
-      <c r="F143">
+      <c r="F145">
         <v>0.1</v>
       </c>
-      <c r="G143" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="144" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A144">
+      <c r="G145" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="146" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A146">
         <v>915</v>
       </c>
-      <c r="B144" t="str">
+      <c r="B146" t="str">
         <f t="shared" si="2"/>
         <v>915</v>
       </c>
-      <c r="C144" t="s">
+      <c r="C146" t="s">
         <v>133</v>
       </c>
-      <c r="D144">
+      <c r="D146">
         <v>9</v>
       </c>
-      <c r="E144" t="s">
+      <c r="E146" t="s">
         <v>130</v>
       </c>
-      <c r="F144">
+      <c r="F146">
         <v>0.1</v>
       </c>
-      <c r="G144" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="145" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A145">
+      <c r="G146" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="147" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A147">
         <v>918</v>
       </c>
-      <c r="B145" t="str">
+      <c r="B147" t="str">
         <f t="shared" si="2"/>
         <v>918</v>
       </c>
-      <c r="C145" t="s">
+      <c r="C147" t="s">
         <v>134</v>
       </c>
-      <c r="D145">
+      <c r="D147">
         <v>9</v>
       </c>
-      <c r="E145" t="s">
+      <c r="E147" t="s">
         <v>130</v>
       </c>
-      <c r="F145">
+      <c r="F147">
         <v>0.1</v>
       </c>
-      <c r="G145" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="146" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A146">
+      <c r="G147" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="148" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A148">
         <v>919</v>
       </c>
-      <c r="B146" t="str">
+      <c r="B148" t="str">
         <f t="shared" si="2"/>
         <v>919</v>
       </c>
-      <c r="C146" t="s">
+      <c r="C148" t="s">
         <v>135</v>
       </c>
-      <c r="D146">
+      <c r="D148">
         <v>9</v>
       </c>
-      <c r="E146" t="s">
+      <c r="E148" t="s">
         <v>130</v>
       </c>
-      <c r="F146">
+      <c r="F148">
         <v>0.1</v>
       </c>
-      <c r="G146" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="147" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A147">
+      <c r="G148" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="149" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A149">
         <v>990</v>
       </c>
-      <c r="B147" t="str">
+      <c r="B149" t="str">
         <f t="shared" si="2"/>
         <v>990</v>
       </c>
-      <c r="C147" t="s">
+      <c r="C149" t="s">
         <v>136</v>
       </c>
-      <c r="D147">
+      <c r="D149">
         <v>9</v>
       </c>
-      <c r="E147" t="s">
+      <c r="E149" t="s">
         <v>130</v>
       </c>
-      <c r="F147">
+      <c r="F149">
         <v>0.1</v>
       </c>
-      <c r="G147" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="148" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A148">
+      <c r="G149" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="150" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A150">
         <v>991</v>
       </c>
-      <c r="B148" t="str">
+      <c r="B150" t="str">
         <f t="shared" si="2"/>
         <v>991</v>
       </c>
-      <c r="C148" t="s">
+      <c r="C150" t="s">
         <v>137</v>
       </c>
-      <c r="D148">
+      <c r="D150">
         <v>9</v>
       </c>
-      <c r="E148" t="s">
+      <c r="E150" t="s">
         <v>130</v>
       </c>
-      <c r="F148">
+      <c r="F150">
         <v>0.1</v>
       </c>
-      <c r="G148" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="149" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A149">
+      <c r="G150" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="151" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A151">
         <v>996</v>
       </c>
-      <c r="B149" t="str">
+      <c r="B151" t="str">
         <f t="shared" si="2"/>
         <v>996</v>
       </c>
-      <c r="C149" t="s">
+      <c r="C151" t="s">
         <v>46</v>
       </c>
-      <c r="D149">
+      <c r="D151">
         <v>9</v>
       </c>
-      <c r="E149" t="s">
+      <c r="E151" t="s">
         <v>130</v>
       </c>
-      <c r="F149">
+      <c r="F151">
         <v>0.1</v>
       </c>
-      <c r="G149" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="150" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A150">
+      <c r="G151" t="s">
+        <v>145</v>
+      </c>
+    </row>
+    <row r="152" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A152">
         <v>997</v>
       </c>
-      <c r="B150" t="str">
+      <c r="B152" t="str">
         <f t="shared" si="2"/>
         <v>997</v>
       </c>
-      <c r="C150" t="s">
+      <c r="C152" t="s">
         <v>47</v>
       </c>
-      <c r="D150">
+      <c r="D152">
         <v>9</v>
       </c>
-      <c r="E150" t="s">
+      <c r="E152" t="s">
         <v>130</v>
       </c>
-      <c r="F150">
+      <c r="F152">
         <v>0.1</v>
       </c>
-      <c r="G150" t="s">
+      <c r="G152" t="s">
         <v>145</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G150" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:G152" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
update district by tax code output
update outputs, no code changes
</commit_message>
<xml_diff>
--- a/resources/property classes.xlsx
+++ b/resources/property classes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cmapil-my.sharepoint.com/personal/abahls_cmap_illinois_gov/Documents/Documents/github_repos/effective_property_tax/resources/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="16" documentId="13_ncr:1_{2A60A013-1040-4DEC-B76C-0C647DD12EE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CB25FC7B-8658-46C7-B506-0720494CE9E0}"/>
+  <xr:revisionPtr revIDLastSave="21" documentId="13_ncr:1_{2A60A013-1040-4DEC-B76C-0C647DD12EE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{21273C65-3E87-4048-876E-EC8C002C0210}"/>
   <bookViews>
-    <workbookView xWindow="-11355" yWindow="-16365" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Cook" sheetId="1" r:id="rId1"/>
@@ -45,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="940" uniqueCount="343">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="942" uniqueCount="344">
   <si>
     <t>overall_class</t>
   </si>
@@ -1074,6 +1074,9 @@
   </si>
   <si>
     <t>Commercial incentive land</t>
+  </si>
+  <si>
+    <t>5000 - Locally Assessed Railroad</t>
   </si>
 </sst>
 </file>
@@ -6053,7 +6056,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:C23"/>
+  <dimension ref="A1:C24"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="35" bestFit="1" customWidth="1"/>
@@ -6084,7 +6087,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" t="str">
-        <f t="shared" ref="A3:A23" si="0">LEFT(B3,2)</f>
+        <f t="shared" ref="A3:A24" si="0">LEFT(B3,2)</f>
         <v>12</v>
       </c>
       <c r="B3" t="s">
@@ -6203,15 +6206,15 @@
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="str">
-        <f t="shared" si="0"/>
-        <v>60</v>
-      </c>
-      <c r="B13" s="5" t="s">
-        <v>328</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>151</v>
+      <c r="A13" t="str">
+        <f t="shared" si="0"/>
+        <v>50</v>
+      </c>
+      <c r="B13" t="s">
+        <v>343</v>
+      </c>
+      <c r="C13" t="s">
+        <v>228</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.3">
@@ -6220,31 +6223,31 @@
         <v>60</v>
       </c>
       <c r="B14" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="4" t="str">
+        <f t="shared" si="0"/>
+        <v>60</v>
+      </c>
+      <c r="B15" s="5" t="s">
         <v>329</v>
       </c>
-      <c r="C14" s="5" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A15" t="str">
-        <f t="shared" si="0"/>
-        <v>61</v>
-      </c>
-      <c r="B15" t="s">
-        <v>330</v>
-      </c>
-      <c r="C15" t="s">
+      <c r="C15" s="5" t="s">
         <v>151</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A16" t="str">
         <f t="shared" si="0"/>
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B16" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C16" t="s">
         <v>151</v>
@@ -6253,10 +6256,10 @@
     <row r="17" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A17" t="str">
         <f t="shared" si="0"/>
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B17" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="C17" t="s">
         <v>151</v>
@@ -6265,22 +6268,22 @@
     <row r="18" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A18" t="str">
         <f t="shared" si="0"/>
-        <v>80</v>
+        <v>63</v>
       </c>
       <c r="B18" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="C18" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A19" t="str">
         <f t="shared" si="0"/>
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B19" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="C19" t="s">
         <v>157</v>
@@ -6289,10 +6292,10 @@
     <row r="20" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A20" t="str">
         <f t="shared" si="0"/>
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B20" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="C20" t="s">
         <v>157</v>
@@ -6301,10 +6304,10 @@
     <row r="21" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A21" t="str">
         <f t="shared" si="0"/>
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B21" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C21" t="s">
         <v>157</v>
@@ -6313,24 +6316,36 @@
     <row r="22" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A22" t="str">
         <f t="shared" si="0"/>
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="B22" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="C22" t="s">
-        <v>188</v>
+        <v>157</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A23" t="str">
         <f t="shared" si="0"/>
+        <v>90</v>
+      </c>
+      <c r="B23" t="s">
+        <v>337</v>
+      </c>
+      <c r="C23" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" t="str">
+        <f t="shared" si="0"/>
         <v>MH</v>
       </c>
-      <c r="B23" t="s">
+      <c r="B24" t="s">
         <v>338</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C24" t="s">
         <v>145</v>
       </c>
     </row>

</xml_diff>